<commit_message>
feat(spatialgcn): sync fresh 6-band SpatialGCN conformal evaluation reports and metrics
Co-authored-by: Claude <claude@anthropic.com>
</commit_message>
<xml_diff>
--- a/Classification/spatialgcn/results/uncertainty_results/conformal_reports_all_models.xlsx
+++ b/Classification/spatialgcn/results/uncertainty_results/conformal_reports_all_models.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="92">
   <si>
     <t>model_name</t>
   </si>
@@ -135,22 +135,19 @@
     <t>timestamp_utc</t>
   </si>
   <si>
-    <t>/content/drive/My Drive/Classification/data/data.csv</t>
-  </si>
-  <si>
-    <t>/content/drive/My Drive/Classification/data/ref.csv</t>
-  </si>
-  <si>
-    <t>/content/drive/My Drive/Classification/spatialgcn/models</t>
-  </si>
-  <si>
-    <t>/content/drive/My Drive/Classification/spatialgcn/results/uncertainty_results</t>
-  </si>
-  <si>
-    <t>/content/drive/My Drive/Classification/spatialgcn/results</t>
-  </si>
-  <si>
-    <t>2026-08-21T05:08:46.874774+00:00</t>
+    <t>/kaggle/input/datasets/daneshselwal/dias-6-bands-data/k001.csv</t>
+  </si>
+  <si>
+    <t>/kaggle/input/datasets/daneshselwal/dias-6-bands-data/k002.csv</t>
+  </si>
+  <si>
+    <t>/kaggle/input</t>
+  </si>
+  <si>
+    <t>/kaggle/working/Classification/spatialgcn/results/uncertainty_results</t>
+  </si>
+  <si>
+    <t>2026-10-11T17:20:03.090690+00:00</t>
   </si>
   <si>
     <t>SplitConformal - SpatialGCN</t>
@@ -1561,7 +1558,7 @@
         <v>0</v>
       </c>
       <c r="I2">
-        <v>1.647651504000009</v>
+        <v>1.217364742000029</v>
       </c>
       <c r="J2">
         <v>0.05</v>
@@ -1596,7 +1593,7 @@
         <v>0</v>
       </c>
       <c r="I3">
-        <v>3.064466891000052</v>
+        <v>1.681150191000029</v>
       </c>
       <c r="J3">
         <v>0.05</v>
@@ -1634,7 +1631,7 @@
         <v>0</v>
       </c>
       <c r="I4">
-        <v>0.7217336969999906</v>
+        <v>0.318860567999991</v>
       </c>
       <c r="J4">
         <v>0.05</v>
@@ -1672,7 +1669,7 @@
         <v>0</v>
       </c>
       <c r="I5">
-        <v>1.700015925000002</v>
+        <v>1.537342009000042</v>
       </c>
       <c r="J5">
         <v>0.05</v>
@@ -1707,7 +1704,7 @@
         <v>0</v>
       </c>
       <c r="I6">
-        <v>1.814477462000013</v>
+        <v>1.332043839999983</v>
       </c>
       <c r="J6">
         <v>0.05</v>
@@ -1779,7 +1776,7 @@
         <v>26</v>
       </c>
       <c r="B7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -1875,7 +1872,7 @@
         <v>36</v>
       </c>
       <c r="B19" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -1890,15 +1887,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="J1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -1968,7 +1965,7 @@
         <v>0</v>
       </c>
       <c r="I5">
-        <v>1.814477462000013</v>
+        <v>1.332043839999983</v>
       </c>
       <c r="J5">
         <v>0.05</v>
@@ -1979,18 +1976,18 @@
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>47</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -2072,18 +2069,18 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>50</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -2091,7 +2088,7 @@
         <v>0</v>
       </c>
       <c r="B21" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C21">
         <v>34443</v>
@@ -2102,7 +2099,7 @@
         <v>1</v>
       </c>
       <c r="B22" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C22">
         <v>8395</v>
@@ -2113,7 +2110,7 @@
         <v>2</v>
       </c>
       <c r="B23" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C23">
         <v>10144</v>
@@ -2124,7 +2121,7 @@
         <v>3</v>
       </c>
       <c r="B24" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C24">
         <v>1196</v>
@@ -2135,13 +2132,13 @@
         <v>4</v>
       </c>
       <c r="B25" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C25">
         <v>1613</v>
       </c>
       <c r="J25" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -2149,7 +2146,7 @@
         <v>5</v>
       </c>
       <c r="B26" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C26">
         <v>1265</v>
@@ -2160,7 +2157,7 @@
         <v>6</v>
       </c>
       <c r="B27" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C27">
         <v>633</v>
@@ -2171,7 +2168,7 @@
         <v>7</v>
       </c>
       <c r="B28" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C28">
         <v>43621</v>
@@ -2179,27 +2176,27 @@
     </row>
     <row r="31" spans="1:10">
       <c r="A31" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="33" spans="1:1">
       <c r="A33">
-        <v>0.8623435928934469</v>
+        <v>0.8623435966409893</v>
       </c>
     </row>
     <row r="49" spans="10:10">
       <c r="J49" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="73" spans="10:10">
       <c r="J73" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -2215,15 +2212,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -2293,7 +2290,7 @@
         <v>0</v>
       </c>
       <c r="I5">
-        <v>1.647651504000009</v>
+        <v>1.217364742000029</v>
       </c>
       <c r="J5">
         <v>0.05</v>
@@ -2304,18 +2301,18 @@
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>47</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -2397,18 +2394,18 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>50</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -2416,10 +2413,10 @@
         <v>0</v>
       </c>
       <c r="B21" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C21">
-        <v>33192</v>
+        <v>33191</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -2427,7 +2424,7 @@
         <v>1</v>
       </c>
       <c r="B22" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C22">
         <v>627</v>
@@ -2438,7 +2435,7 @@
         <v>2</v>
       </c>
       <c r="B23" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C23">
         <v>10448</v>
@@ -2449,7 +2446,7 @@
         <v>3</v>
       </c>
       <c r="B24" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C24">
         <v>1180</v>
@@ -2460,13 +2457,13 @@
         <v>4</v>
       </c>
       <c r="B25" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C25">
         <v>1631</v>
       </c>
       <c r="J25" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -2474,7 +2471,7 @@
         <v>5</v>
       </c>
       <c r="B26" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C26">
         <v>789</v>
@@ -2485,7 +2482,7 @@
         <v>6</v>
       </c>
       <c r="B27" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C27">
         <v>140</v>
@@ -2496,23 +2493,23 @@
         <v>7</v>
       </c>
       <c r="B28" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C28">
-        <v>53303</v>
+        <v>53304</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -2520,7 +2517,7 @@
         <v>0</v>
       </c>
       <c r="B33">
-        <v>0.505713164806366</v>
+        <v>0.5057131477926682</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -2528,7 +2525,7 @@
         <v>1</v>
       </c>
       <c r="B34">
-        <v>0.8650865878709458</v>
+        <v>0.8650865476907845</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -2536,7 +2533,7 @@
         <v>2</v>
       </c>
       <c r="B35">
-        <v>0.8363144794468741</v>
+        <v>0.8363145172903725</v>
       </c>
     </row>
     <row r="36" spans="1:2">
@@ -2544,7 +2541,7 @@
         <v>3</v>
       </c>
       <c r="B36">
-        <v>0.9391544439864117</v>
+        <v>0.9391544140560334</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -2552,7 +2549,7 @@
         <v>4</v>
       </c>
       <c r="B37">
-        <v>0.9719925531542389</v>
+        <v>0.9719925520349869</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -2560,7 +2557,7 @@
         <v>5</v>
       </c>
       <c r="B38">
-        <v>0.9491665584225357</v>
+        <v>0.9491665409086293</v>
       </c>
     </row>
     <row r="39" spans="1:2">
@@ -2568,17 +2565,17 @@
         <v>6</v>
       </c>
       <c r="B39">
-        <v>0.9365353891769739</v>
+        <v>0.9365353863431057</v>
       </c>
     </row>
     <row r="49" spans="10:10">
       <c r="J49" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="73" spans="10:10">
       <c r="J73" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -2594,15 +2591,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="J1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -2672,7 +2669,7 @@
         <v>0</v>
       </c>
       <c r="I5">
-        <v>1.700015925000002</v>
+        <v>1.537342009000042</v>
       </c>
       <c r="J5">
         <v>0.05</v>
@@ -2683,18 +2680,18 @@
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>47</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -2776,18 +2773,18 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>50</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -2795,7 +2792,7 @@
         <v>0</v>
       </c>
       <c r="B21" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C21">
         <v>31768</v>
@@ -2806,7 +2803,7 @@
         <v>1</v>
       </c>
       <c r="B22" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C22">
         <v>114</v>
@@ -2817,7 +2814,7 @@
         <v>2</v>
       </c>
       <c r="B23" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C23">
         <v>8763</v>
@@ -2828,7 +2825,7 @@
         <v>3</v>
       </c>
       <c r="B24" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C24">
         <v>561</v>
@@ -2839,13 +2836,13 @@
         <v>4</v>
       </c>
       <c r="B25" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C25">
         <v>1449</v>
       </c>
       <c r="J25" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -2853,7 +2850,7 @@
         <v>5</v>
       </c>
       <c r="B26" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C26">
         <v>737</v>
@@ -2864,7 +2861,7 @@
         <v>6</v>
       </c>
       <c r="B27" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C27">
         <v>1</v>
@@ -2875,7 +2872,7 @@
         <v>7</v>
       </c>
       <c r="B28" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C28">
         <v>57917</v>
@@ -2883,18 +2880,18 @@
     </row>
     <row r="31" spans="1:10">
       <c r="A31" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B32" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C32" s="1" t="s">
         <v>70</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -2902,7 +2899,7 @@
         <v>0</v>
       </c>
       <c r="B33">
-        <v>0.5649026251026996</v>
+        <v>0.5649025782813054</v>
       </c>
       <c r="C33">
         <v>1</v>
@@ -2913,7 +2910,7 @@
         <v>1</v>
       </c>
       <c r="B34">
-        <v>0.8959801331047826</v>
+        <v>0.8959802021459666</v>
       </c>
       <c r="C34">
         <v>2</v>
@@ -2924,7 +2921,7 @@
         <v>2</v>
       </c>
       <c r="B35">
-        <v>0.8748926743928984</v>
+        <v>0.8748927030300666</v>
       </c>
       <c r="C35">
         <v>2</v>
@@ -2935,7 +2932,7 @@
         <v>3</v>
       </c>
       <c r="B36">
-        <v>0.9392779011216169</v>
+        <v>0.9392779023092059</v>
       </c>
       <c r="C36">
         <v>4</v>
@@ -2946,7 +2943,7 @@
         <v>4</v>
       </c>
       <c r="B37">
-        <v>0.9729664923145289</v>
+        <v>0.9729664917107296</v>
       </c>
       <c r="C37">
         <v>4</v>
@@ -2957,7 +2954,7 @@
         <v>5</v>
       </c>
       <c r="B38">
-        <v>0.9778143710318206</v>
+        <v>0.97781438392877</v>
       </c>
       <c r="C38">
         <v>4</v>
@@ -2968,7 +2965,7 @@
         <v>6</v>
       </c>
       <c r="B39">
-        <v>0.9365353891769739</v>
+        <v>0.9365353863431057</v>
       </c>
       <c r="C39">
         <v>3</v>
@@ -2976,12 +2973,12 @@
     </row>
     <row r="49" spans="10:10">
       <c r="J49" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="73" spans="10:10">
       <c r="J73" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -2997,15 +2994,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -3075,7 +3072,7 @@
         <v>0</v>
       </c>
       <c r="I5">
-        <v>3.064466891000052</v>
+        <v>1.681150191000029</v>
       </c>
       <c r="J5">
         <v>0.05</v>
@@ -3089,18 +3086,18 @@
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>47</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -3182,15 +3179,15 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -3233,7 +3230,7 @@
         <v>2</v>
       </c>
       <c r="J25" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -3254,15 +3251,15 @@
     </row>
     <row r="30" spans="1:10">
       <c r="A30" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="32" spans="1:10">
@@ -3270,7 +3267,7 @@
         <v>0</v>
       </c>
       <c r="B32">
-        <v>0.8233219912808597</v>
+        <v>0.8233220280862208</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -3278,7 +3275,7 @@
         <v>1</v>
       </c>
       <c r="B33">
-        <v>0.9365353891769739</v>
+        <v>0.9365353863431057</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -3286,7 +3283,7 @@
         <v>2</v>
       </c>
       <c r="B34">
-        <v>0.9719925531542389</v>
+        <v>0.9719925520349869</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -3294,20 +3291,20 @@
         <v>3</v>
       </c>
       <c r="B35">
-        <v>0.9491665584225357</v>
+        <v>0.9491665409086293</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B39" s="1" t="s">
         <v>78</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="40" spans="1:2">
@@ -3344,15 +3341,15 @@
     </row>
     <row r="46" spans="1:2">
       <c r="A46" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -3371,7 +3368,7 @@
         <v>0.389937106918239</v>
       </c>
       <c r="J49" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="50" spans="1:10">
@@ -3416,7 +3413,7 @@
     </row>
     <row r="73" spans="10:10">
       <c r="J73" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -3432,15 +3429,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -3510,7 +3507,7 @@
         <v>0</v>
       </c>
       <c r="I5">
-        <v>0.7217336969999906</v>
+        <v>0.318860567999991</v>
       </c>
       <c r="J5">
         <v>0.05</v>
@@ -3524,18 +3521,18 @@
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>47</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -3617,23 +3614,23 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="C20" s="1" t="s">
         <v>87</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21">
-        <v>0.7643444223054584</v>
+        <v>0.7643443955354527</v>
       </c>
       <c r="B21">
         <v>0.01</v>
@@ -3655,7 +3652,7 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -3739,12 +3736,12 @@
     </row>
     <row r="13" spans="1:13">
       <c r="A13" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="41" spans="1:1">
       <c r="A41" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -3760,7 +3757,7 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -3844,12 +3841,12 @@
     </row>
     <row r="13" spans="1:13">
       <c r="A13" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="41" spans="1:1">
       <c r="A41" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>

</xml_diff>